<commit_message>
Team-Liste: Rollen pro Folie, optional zweite Person, Zeit je Person
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111joxY9HLNj7w7Z5tgi3FM
</commit_message>
<xml_diff>
--- a/endpraesentation/Team_Leitfaden_Elbharz.xlsx
+++ b/endpraesentation/Team_Leitfaden_Elbharz.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="164">
   <si>
     <t xml:space="preserve">Team-Leitfaden Endpräsentation – Elbharz Getränke GbR</t>
   </si>
@@ -74,7 +74,7 @@
     <t xml:space="preserve">Blatt „Rollen &amp; Zeitplan“</t>
   </si>
   <si>
-    <t xml:space="preserve">Wer spricht welche Folie – Namen auswählen. Die Zeiten rechnen sich mit.</t>
+    <t xml:space="preserve">Jede Folie einzeln vergeben, auch abwechselnd; optional eine 2. Person pro Folie. Zeit und Anzahl Folien je Person rechnen sich mit.</t>
   </si>
   <si>
     <t xml:space="preserve">Blatt „Sprechtexte“</t>
@@ -260,7 +260,7 @@
     <t xml:space="preserve">Rollen &amp; Zeitplan</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprecher:in je Folie auswählen. Vorschlag: Person 1 = Folien 1–4, Person 2 = 5–6, Person 3 = 7–9, Person 4 = 10–12.</t>
+    <t xml:space="preserve">Jede Folie einzeln vergeben – gern abwechselnd. Teilen sich zwei eine Folie, zweite Person eintragen: die Zeit wird halbiert.</t>
   </si>
   <si>
     <t xml:space="preserve">Folie</t>
@@ -275,12 +275,18 @@
     <t xml:space="preserve">Sprecher:in</t>
   </si>
   <si>
+    <t xml:space="preserve">2. Sprecher:in (optional)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dauer</t>
   </si>
   <si>
     <t xml:space="preserve">bis (Stoppuhr)</t>
   </si>
   <si>
+    <t xml:space="preserve">Übergabe / Notiz</t>
+  </si>
+  <si>
     <t xml:space="preserve">Primatenbrause (Titel)</t>
   </si>
   <si>
@@ -335,10 +341,22 @@
     <t xml:space="preserve">Summe Sprechzeit (ohne Wechsel)</t>
   </si>
   <si>
-    <t xml:space="preserve">Zeit je Person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grenze laut Aufgabe: 10–12 Minuten. Mit Sprecherwechseln etwa 20–30 Sekunden mehr einplanen.</t>
+    <t xml:space="preserve">Folien ohne Sprecher:in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeit und Folien je Person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grenze laut Aufgabe: 10–12 Minuten. Pro Sprecherwechsel etwa 5 Sekunden mehr einplanen – viele Wechsel kosten Zeit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faustregel: Wechsel an Kapitelgrenzen wirken ruhiger; ein Wechsel mitten in einer Folie braucht einen klaren Übergabesatz (Spalte H).</t>
   </si>
   <si>
     <t xml:space="preserve">Sprechtexte</t>
@@ -507,12 +525,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="166" formatCode="[m]:ss"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -613,6 +632,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFD9822B"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="11"/>
       <color rgb="FF5F8F99"/>
@@ -690,7 +717,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -775,11 +802,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1134,7 +1165,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
         <v>14</v>
       </c>
@@ -1764,15 +1795,16 @@
     <tabColor rgb="FF8DB33A"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1785,7 +1817,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
         <v>78</v>
       </c>
@@ -1803,6 +1835,12 @@
       </c>
       <c r="F4" s="12" t="s">
         <v>83</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1810,291 +1848,351 @@
         <v>1</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D5" s="16"/>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="16"/>
+      <c r="F5" s="19" t="n">
         <v>0.000231481481481482</v>
       </c>
-      <c r="F5" s="19" t="n">
-        <f aca="false">SUM($E$5:E5)</f>
+      <c r="G5" s="19" t="n">
+        <f aca="false">SUM($F$5:F5)</f>
         <v>0.000231481481481482</v>
       </c>
+      <c r="H5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D6" s="16"/>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="16"/>
+      <c r="F6" s="19" t="n">
         <v>0.000520833333333333</v>
       </c>
-      <c r="F6" s="19" t="n">
-        <f aca="false">SUM($E$5:E6)</f>
+      <c r="G6" s="19" t="n">
+        <f aca="false">SUM($F$5:F6)</f>
         <v>0.000752314814814815</v>
       </c>
+      <c r="H6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D7" s="16"/>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="16"/>
+      <c r="F7" s="19" t="n">
         <v>0.000520833333333333</v>
       </c>
-      <c r="F7" s="19" t="n">
-        <f aca="false">SUM($E$5:E7)</f>
+      <c r="G7" s="19" t="n">
+        <f aca="false">SUM($F$5:F7)</f>
         <v>0.00127314814814815</v>
       </c>
+      <c r="H7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D8" s="16"/>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="16"/>
+      <c r="F8" s="19" t="n">
         <v>0.000694444444444445</v>
       </c>
-      <c r="F8" s="19" t="n">
-        <f aca="false">SUM($E$5:E8)</f>
+      <c r="G8" s="19" t="n">
+        <f aca="false">SUM($F$5:F8)</f>
         <v>0.00196759259259259</v>
       </c>
+      <c r="H8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D9" s="16"/>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="16"/>
+      <c r="F9" s="19" t="n">
         <v>0.000752314814814815</v>
       </c>
-      <c r="F9" s="19" t="n">
-        <f aca="false">SUM($E$5:E9)</f>
+      <c r="G9" s="19" t="n">
+        <f aca="false">SUM($F$5:F9)</f>
         <v>0.00271990740740741</v>
       </c>
+      <c r="H9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>90</v>
-      </c>
       <c r="D10" s="16"/>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="16"/>
+      <c r="F10" s="19" t="n">
         <v>0.000578703703703704</v>
       </c>
-      <c r="F10" s="19" t="n">
-        <f aca="false">SUM($E$5:E10)</f>
+      <c r="G10" s="19" t="n">
+        <f aca="false">SUM($F$5:F10)</f>
         <v>0.00329861111111111</v>
       </c>
+      <c r="H10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D11" s="16"/>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="16"/>
+      <c r="F11" s="19" t="n">
         <v>0.000694444444444445</v>
       </c>
-      <c r="F11" s="19" t="n">
-        <f aca="false">SUM($E$5:E11)</f>
+      <c r="G11" s="19" t="n">
+        <f aca="false">SUM($F$5:F11)</f>
         <v>0.00399305555555556</v>
       </c>
+      <c r="H11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D12" s="16"/>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="16"/>
+      <c r="F12" s="19" t="n">
         <v>0.000636574074074074</v>
       </c>
-      <c r="F12" s="19" t="n">
-        <f aca="false">SUM($E$5:E12)</f>
+      <c r="G12" s="19" t="n">
+        <f aca="false">SUM($F$5:F12)</f>
         <v>0.00462962962962963</v>
       </c>
+      <c r="H12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="C13" s="14" t="s">
-        <v>94</v>
-      </c>
       <c r="D13" s="16"/>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="16"/>
+      <c r="F13" s="19" t="n">
         <v>0.000578703703703704</v>
       </c>
-      <c r="F13" s="19" t="n">
-        <f aca="false">SUM($E$5:E13)</f>
+      <c r="G13" s="19" t="n">
+        <f aca="false">SUM($F$5:F13)</f>
         <v>0.00520833333333333</v>
       </c>
+      <c r="H13" s="16"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D14" s="16"/>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="16"/>
+      <c r="F14" s="19" t="n">
         <v>0.000925925925925926</v>
       </c>
-      <c r="F14" s="19" t="n">
-        <f aca="false">SUM($E$5:E14)</f>
+      <c r="G14" s="19" t="n">
+        <f aca="false">SUM($F$5:F14)</f>
         <v>0.00613425925925926</v>
       </c>
+      <c r="H14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D15" s="16"/>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="16"/>
+      <c r="F15" s="19" t="n">
         <v>0.000810185185185185</v>
       </c>
-      <c r="F15" s="19" t="n">
-        <f aca="false">SUM($E$5:E15)</f>
+      <c r="G15" s="19" t="n">
+        <f aca="false">SUM($F$5:F15)</f>
         <v>0.00694444444444444</v>
       </c>
+      <c r="H15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D16" s="16"/>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="16"/>
+      <c r="F16" s="19" t="n">
         <v>0.000115740740740741</v>
       </c>
-      <c r="F16" s="19" t="n">
-        <f aca="false">SUM($E$5:E16)</f>
+      <c r="G16" s="19" t="n">
+        <f aca="false">SUM($F$5:F16)</f>
         <v>0.00706018518518519</v>
       </c>
+      <c r="H16" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="E18" s="20" t="n">
-        <f aca="false">SUM(E5:E16)</f>
+        <v>103</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <f aca="false">SUM(F5:F16)</f>
         <v>0.00706018518518519</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="10" t="s">
-        <v>102</v>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <f aca="false">COUNTBLANK(D5:D16)</f>
+        <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="str">
+      <c r="B21" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4" t="str">
         <f aca="false">IF(Start!$B$5="","Person 1",Start!$B$5)</f>
         <v>Person 1</v>
       </c>
-      <c r="E21" s="21" t="n">
-        <f aca="false">SUMIF($D$5:$D$16,Start!$B$5,$E$5:$E$16)</f>
+      <c r="D22" s="4" t="n">
+        <f aca="false">IF(Start!$B$5="",0,COUNTIF($D$5:$D$16,Start!$B$5)+COUNTIF($E$5:$E$16,Start!$B$5))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="4" t="str">
+      <c r="F22" s="22" t="n">
+        <f aca="false">IF(Start!$B$5="",0,SUMPRODUCT((($D$5:$D$16=Start!$B$5)+($E$5:$E$16=Start!$B$5))*$F$5:$F$16/(($E$5:$E$16&lt;&gt;"")+1)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="4" t="str">
         <f aca="false">IF(Start!$B$6="","Person 2",Start!$B$6)</f>
         <v>Person 2</v>
       </c>
-      <c r="E22" s="21" t="n">
-        <f aca="false">SUMIF($D$5:$D$16,Start!$B$6,$E$5:$E$16)</f>
+      <c r="D23" s="4" t="n">
+        <f aca="false">IF(Start!$B$6="",0,COUNTIF($D$5:$D$16,Start!$B$6)+COUNTIF($E$5:$E$16,Start!$B$6))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="4" t="str">
+      <c r="F23" s="22" t="n">
+        <f aca="false">IF(Start!$B$6="",0,SUMPRODUCT((($D$5:$D$16=Start!$B$6)+($E$5:$E$16=Start!$B$6))*$F$5:$F$16/(($E$5:$E$16&lt;&gt;"")+1)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="str">
         <f aca="false">IF(Start!$B$7="","Person 3",Start!$B$7)</f>
         <v>Person 3</v>
       </c>
-      <c r="E23" s="21" t="n">
-        <f aca="false">SUMIF($D$5:$D$16,Start!$B$7,$E$5:$E$16)</f>
+      <c r="D24" s="4" t="n">
+        <f aca="false">IF(Start!$B$7="",0,COUNTIF($D$5:$D$16,Start!$B$7)+COUNTIF($E$5:$E$16,Start!$B$7))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="4" t="str">
+      <c r="F24" s="22" t="n">
+        <f aca="false">IF(Start!$B$7="",0,SUMPRODUCT((($D$5:$D$16=Start!$B$7)+($E$5:$E$16=Start!$B$7))*$F$5:$F$16/(($E$5:$E$16&lt;&gt;"")+1)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="4" t="str">
         <f aca="false">IF(Start!$B$8="","Person 4",Start!$B$8)</f>
         <v>Person 4</v>
       </c>
-      <c r="E24" s="21" t="n">
-        <f aca="false">SUMIF($D$5:$D$16,Start!$B$8,$E$5:$E$16)</f>
+      <c r="D25" s="4" t="n">
+        <f aca="false">IF(Start!$B$8="",0,COUNTIF($D$5:$D$16,Start!$B$8)+COUNTIF($E$5:$E$16,Start!$B$8))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="22" t="s">
-        <v>103</v>
+      <c r="F25" s="22" t="n">
+        <f aca="false">IF(Start!$B$8="",0,SUMPRODUCT((($D$5:$D$16=Start!$B$8)+($E$5:$E$16=Start!$B$8))*$F$5:$F$16/(($E$5:$E$16&lt;&gt;"")+1)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="23" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="23" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:E16" type="list">
       <formula1>Team</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2126,12 +2224,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2142,167 +2240,167 @@
         <v>81</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="n">
+      <c r="A5" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D5</f>
-        <v>0</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" s="24"/>
+      <c r="B5" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D5="","",IF('Rollen &amp; Zeitplan'!E5="",'Rollen &amp; Zeitplan'!D5,'Rollen &amp; Zeitplan'!D5&amp;" + "&amp;'Rollen &amp; Zeitplan'!E5))</f>
+        <v/>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="n">
+      <c r="A6" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D6</f>
-        <v>0</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>109</v>
-      </c>
-      <c r="D6" s="24"/>
+      <c r="B6" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D6="","",IF('Rollen &amp; Zeitplan'!E6="",'Rollen &amp; Zeitplan'!D6,'Rollen &amp; Zeitplan'!D6&amp;" + "&amp;'Rollen &amp; Zeitplan'!E6))</f>
+        <v/>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="n">
+      <c r="A7" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D7</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="D7" s="24"/>
+      <c r="B7" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D7="","",IF('Rollen &amp; Zeitplan'!E7="",'Rollen &amp; Zeitplan'!D7,'Rollen &amp; Zeitplan'!D7&amp;" + "&amp;'Rollen &amp; Zeitplan'!E7))</f>
+        <v/>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="n">
+      <c r="A8" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D8</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="D8" s="24"/>
+      <c r="B8" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D8="","",IF('Rollen &amp; Zeitplan'!E8="",'Rollen &amp; Zeitplan'!D8,'Rollen &amp; Zeitplan'!D8&amp;" + "&amp;'Rollen &amp; Zeitplan'!E8))</f>
+        <v/>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="n">
+      <c r="A9" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D9</f>
-        <v>0</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="D9" s="24"/>
+      <c r="B9" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D9="","",IF('Rollen &amp; Zeitplan'!E9="",'Rollen &amp; Zeitplan'!D9,'Rollen &amp; Zeitplan'!D9&amp;" + "&amp;'Rollen &amp; Zeitplan'!E9))</f>
+        <v/>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
+      <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D10</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="D10" s="24"/>
+      <c r="B10" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D10="","",IF('Rollen &amp; Zeitplan'!E10="",'Rollen &amp; Zeitplan'!D10,'Rollen &amp; Zeitplan'!D10&amp;" + "&amp;'Rollen &amp; Zeitplan'!E10))</f>
+        <v/>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="n">
+      <c r="A11" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D11</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="D11" s="24"/>
+      <c r="B11" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D11="","",IF('Rollen &amp; Zeitplan'!E11="",'Rollen &amp; Zeitplan'!D11,'Rollen &amp; Zeitplan'!D11&amp;" + "&amp;'Rollen &amp; Zeitplan'!E11))</f>
+        <v/>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="24" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D12</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="D12" s="24"/>
+      <c r="B12" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D12="","",IF('Rollen &amp; Zeitplan'!E12="",'Rollen &amp; Zeitplan'!D12,'Rollen &amp; Zeitplan'!D12&amp;" + "&amp;'Rollen &amp; Zeitplan'!E12))</f>
+        <v/>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="n">
+      <c r="A13" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D13</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="D13" s="24"/>
+      <c r="B13" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D13="","",IF('Rollen &amp; Zeitplan'!E13="",'Rollen &amp; Zeitplan'!D13,'Rollen &amp; Zeitplan'!D13&amp;" + "&amp;'Rollen &amp; Zeitplan'!E13))</f>
+        <v/>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="n">
+      <c r="A14" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D14</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="D14" s="24"/>
+      <c r="B14" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D14="","",IF('Rollen &amp; Zeitplan'!E14="",'Rollen &amp; Zeitplan'!D14,'Rollen &amp; Zeitplan'!D14&amp;" + "&amp;'Rollen &amp; Zeitplan'!E14))</f>
+        <v/>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="25"/>
     </row>
     <row r="15" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="n">
+      <c r="A15" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D15</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="D15" s="24"/>
+      <c r="B15" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D15="","",IF('Rollen &amp; Zeitplan'!E15="",'Rollen &amp; Zeitplan'!D15,'Rollen &amp; Zeitplan'!D15&amp;" + "&amp;'Rollen &amp; Zeitplan'!E15))</f>
+        <v/>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="D15" s="25"/>
     </row>
     <row r="16" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="n">
+      <c r="A16" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="23" t="n">
-        <f aca="false">'Rollen &amp; Zeitplan'!D16</f>
-        <v>0</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D16" s="24"/>
+      <c r="B16" s="24" t="str">
+        <f aca="false">IF('Rollen &amp; Zeitplan'!D16="","",IF('Rollen &amp; Zeitplan'!E16="",'Rollen &amp; Zeitplan'!D16,'Rollen &amp; Zeitplan'!D16&amp;" + "&amp;'Rollen &amp; Zeitplan'!E16))</f>
+        <v/>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="D16" s="25"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2332,159 +2430,159 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="D5" s="24"/>
+      <c r="A5" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="D6" s="24"/>
+      <c r="A6" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="D7" s="24"/>
+      <c r="A7" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>135</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="D8" s="24"/>
+      <c r="A8" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
-        <v>138</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="D9" s="24"/>
+      <c r="A9" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>141</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="D10" s="24"/>
+      <c r="A10" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="D11" s="24"/>
+      <c r="A11" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="D12" s="24"/>
+      <c r="A12" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
-        <v>150</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="D13" s="24"/>
+      <c r="A13" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>157</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="D14" s="24"/>
+      <c r="A14" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="D14" s="25"/>
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>156</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="24"/>
+      <c r="A15" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="25"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Teamnamen in Excel-Liste vorbelegt, Bilder komprimiert (Präsentation 361 KB)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111joxY9HLNj7w7Z5tgi3FM
</commit_message>
<xml_diff>
--- a/endpraesentation/Team_Leitfaden_Elbharz.xlsx
+++ b/endpraesentation/Team_Leitfaden_Elbharz.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="168">
   <si>
     <t xml:space="preserve">Team-Leitfaden Endpräsentation – Elbharz Getränke GbR</t>
   </si>
@@ -35,19 +35,31 @@
     <t xml:space="preserve">Gemeinsam in OneDrive/SharePoint öffnen – alle können gleichzeitig bearbeiten.</t>
   </si>
   <si>
-    <t xml:space="preserve">Unsere Namen (hier eintragen – erscheinen dann überall als Spalten und in den Auswahllisten):</t>
+    <t xml:space="preserve">Unsere Namen (erscheinen überall als Spalten und in den Auswahllisten – nur hier ändern):</t>
   </si>
   <si>
     <t xml:space="preserve">Person 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Jona</t>
+  </si>
+  <si>
     <t xml:space="preserve">Person 2</t>
   </si>
   <si>
+    <t xml:space="preserve">Lennart</t>
+  </si>
+  <si>
     <t xml:space="preserve">Person 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Sönke</t>
+  </si>
+  <si>
     <t xml:space="preserve">Person 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nio</t>
   </si>
   <si>
     <t xml:space="preserve">So funktioniert's</t>
@@ -1115,83 +1127,91 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5"/>
+      <c r="B5" s="5" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="5"/>
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="5"/>
+        <v>7</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5"/>
+        <v>9</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B19" s="10" t="str">
         <f aca="false">Aufgaben!B3</f>
@@ -1230,12 +1250,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1246,37 +1266,37 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D6" s="13" t="str">
         <f aca="false">IF(Start!$B$5="","Person 1",Start!$B$5)</f>
-        <v>Person 1</v>
+        <v>Jona</v>
       </c>
       <c r="E6" s="13" t="str">
         <f aca="false">IF(Start!$B$6="","Person 2",Start!$B$6)</f>
-        <v>Person 2</v>
+        <v>Lennart</v>
       </c>
       <c r="F6" s="13" t="str">
         <f aca="false">IF(Start!$B$7="","Person 3",Start!$B$7)</f>
-        <v>Person 3</v>
+        <v>Sönke</v>
       </c>
       <c r="G6" s="13" t="str">
         <f aca="false">IF(Start!$B$8="","Person 4",Start!$B$8)</f>
-        <v>Person 4</v>
+        <v>Nio</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1284,10 +1304,10 @@
         <v>1</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
@@ -1303,10 +1323,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
@@ -1322,10 +1342,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D9" s="15"/>
       <c r="E9" s="15"/>
@@ -1341,10 +1361,10 @@
         <v>4</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
@@ -1360,10 +1380,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="15"/>
@@ -1379,10 +1399,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
@@ -1398,10 +1418,10 @@
         <v>7</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
@@ -1414,30 +1434,30 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="H17" s="12"/>
     </row>
@@ -1446,10 +1466,10 @@
         <v>1</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D18" s="16"/>
       <c r="E18" s="17"/>
@@ -1465,10 +1485,10 @@
         <v>2</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D19" s="16"/>
       <c r="E19" s="17"/>
@@ -1484,10 +1504,10 @@
         <v>3</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="17"/>
@@ -1503,10 +1523,10 @@
         <v>4</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D21" s="16"/>
       <c r="E21" s="17"/>
@@ -1522,10 +1542,10 @@
         <v>5</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D22" s="16"/>
       <c r="E22" s="17"/>
@@ -1541,10 +1561,10 @@
         <v>6</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="17"/>
@@ -1560,10 +1580,10 @@
         <v>7</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D24" s="16"/>
       <c r="E24" s="17"/>
@@ -1579,10 +1599,10 @@
         <v>8</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D25" s="16"/>
       <c r="E25" s="17"/>
@@ -1598,10 +1618,10 @@
         <v>9</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D26" s="16"/>
       <c r="E26" s="17"/>
@@ -1617,10 +1637,10 @@
         <v>10</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="17"/>
@@ -1636,10 +1656,10 @@
         <v>11</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="17"/>
@@ -1655,10 +1675,10 @@
         <v>12</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="17"/>
@@ -1674,10 +1694,10 @@
         <v>13</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="17"/>
@@ -1693,10 +1713,10 @@
         <v>14</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="17"/>
@@ -1712,10 +1732,10 @@
         <v>15</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="17"/>
@@ -1809,38 +1829,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1848,10 +1868,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -1869,10 +1889,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -1890,10 +1910,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -1911,10 +1931,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
@@ -1932,10 +1952,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -1953,10 +1973,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
@@ -1974,10 +1994,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
@@ -1995,10 +2015,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
@@ -2016,10 +2036,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
@@ -2037,10 +2057,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -2058,10 +2078,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
@@ -2079,10 +2099,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
@@ -2097,7 +2117,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F18" s="20" t="n">
         <f aca="false">SUM(F5:F16)</f>
@@ -2106,7 +2126,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="9" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F19" s="21" t="n">
         <f aca="false">COUNTBLANK(D5:D16)</f>
@@ -2115,19 +2135,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="10" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="4" t="str">
         <f aca="false">IF(Start!$B$5="","Person 1",Start!$B$5)</f>
-        <v>Person 1</v>
+        <v>Jona</v>
       </c>
       <c r="D22" s="4" t="n">
         <f aca="false">IF(Start!$B$5="",0,COUNTIF($D$5:$D$16,Start!$B$5)+COUNTIF($E$5:$E$16,Start!$B$5))</f>
@@ -2141,7 +2161,7 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="4" t="str">
         <f aca="false">IF(Start!$B$6="","Person 2",Start!$B$6)</f>
-        <v>Person 2</v>
+        <v>Lennart</v>
       </c>
       <c r="D23" s="4" t="n">
         <f aca="false">IF(Start!$B$6="",0,COUNTIF($D$5:$D$16,Start!$B$6)+COUNTIF($E$5:$E$16,Start!$B$6))</f>
@@ -2155,7 +2175,7 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="4" t="str">
         <f aca="false">IF(Start!$B$7="","Person 3",Start!$B$7)</f>
-        <v>Person 3</v>
+        <v>Sönke</v>
       </c>
       <c r="D24" s="4" t="n">
         <f aca="false">IF(Start!$B$7="",0,COUNTIF($D$5:$D$16,Start!$B$7)+COUNTIF($E$5:$E$16,Start!$B$7))</f>
@@ -2169,7 +2189,7 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="4" t="str">
         <f aca="false">IF(Start!$B$8="","Person 4",Start!$B$8)</f>
-        <v>Person 4</v>
+        <v>Nio</v>
       </c>
       <c r="D25" s="4" t="n">
         <f aca="false">IF(Start!$B$8="",0,COUNTIF($D$5:$D$16,Start!$B$8)+COUNTIF($E$5:$E$16,Start!$B$8))</f>
@@ -2182,12 +2202,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="23" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="23" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2224,26 +2244,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2255,7 +2275,7 @@
         <v/>
       </c>
       <c r="C5" s="24" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D5" s="25"/>
     </row>
@@ -2268,7 +2288,7 @@
         <v/>
       </c>
       <c r="C6" s="24" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D6" s="25"/>
     </row>
@@ -2281,7 +2301,7 @@
         <v/>
       </c>
       <c r="C7" s="24" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D7" s="25"/>
     </row>
@@ -2294,7 +2314,7 @@
         <v/>
       </c>
       <c r="C8" s="24" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D8" s="25"/>
     </row>
@@ -2307,7 +2327,7 @@
         <v/>
       </c>
       <c r="C9" s="24" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D9" s="25"/>
     </row>
@@ -2320,7 +2340,7 @@
         <v/>
       </c>
       <c r="C10" s="24" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D10" s="25"/>
     </row>
@@ -2333,7 +2353,7 @@
         <v/>
       </c>
       <c r="C11" s="24" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D11" s="25"/>
     </row>
@@ -2346,7 +2366,7 @@
         <v/>
       </c>
       <c r="C12" s="24" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D12" s="25"/>
     </row>
@@ -2359,7 +2379,7 @@
         <v/>
       </c>
       <c r="C13" s="24" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D13" s="25"/>
     </row>
@@ -2372,7 +2392,7 @@
         <v/>
       </c>
       <c r="C14" s="24" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D14" s="25"/>
     </row>
@@ -2385,7 +2405,7 @@
         <v/>
       </c>
       <c r="C15" s="24" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D15" s="25"/>
     </row>
@@ -2398,7 +2418,7 @@
         <v/>
       </c>
       <c r="C16" s="24" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D16" s="25"/>
     </row>
@@ -2430,157 +2450,157 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D5" s="25"/>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D6" s="25"/>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D7" s="25"/>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D9" s="25"/>
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D11" s="25"/>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D12" s="25"/>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D14" s="25"/>
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="26" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D15" s="25"/>
     </row>

</xml_diff>

<commit_message>
Version 2: Feedback umgesetzt (Reihenfolge, 3 Entscheidungen, Kennzahlen schlank, Schluss-Bogen, Anhang), Sprechtext als Word, Excel aktualisiert
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111joxY9HLNj7w7Z5tgi3FM
</commit_message>
<xml_diff>
--- a/endpraesentation/Team_Leitfaden_Elbharz.xlsx
+++ b/endpraesentation/Team_Leitfaden_Elbharz.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
   <si>
     <t xml:space="preserve">Elbharz · Aufgaben bis zur Präsentation</t>
   </si>
@@ -50,10 +50,10 @@
     <t xml:space="preserve">Nio</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprechtext für meine Folien in eigene Worte gebracht</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meinen Teil laut mit Stoppuhr geübt</t>
+    <t xml:space="preserve">Sprechtext für meine Folien gelesen und in eigene Worte gebracht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meinen Teil laut mit Stoppuhr geübt (inkl. Übergabesatz)</t>
   </si>
   <si>
     <t xml:space="preserve">Kann die Zahlen meiner Folien ohne Ablesen erklären</t>
@@ -74,7 +74,7 @@
     <t xml:space="preserve">Erledigt von</t>
   </si>
   <si>
-    <t xml:space="preserve">Karte Norddeutschland mit roter Elbe einfügen (Folie 3)</t>
+    <t xml:space="preserve">Optional: Karte mit roter Elbe statt Standort-Symbol (Folie 3)</t>
   </si>
   <si>
     <t xml:space="preserve">KI-Teambild einfügen + Tool notieren (Folie 12)</t>
@@ -101,7 +101,7 @@
     <t xml:space="preserve">Wer spricht was</t>
   </si>
   <si>
-    <t xml:space="preserve">Pro Folie einen Namen wählen – Wechsel sind jederzeit möglich.</t>
+    <t xml:space="preserve">Pro Folie einen Namen wählen. Vorschlag: Folie 1–3 · 4–6 · 7–9 · 10–12 (passt zu den Kapiteln).</t>
   </si>
   <si>
     <t xml:space="preserve">Folie</t>
@@ -116,6 +116,9 @@
     <t xml:space="preserve">Dauer</t>
   </si>
   <si>
+    <t xml:space="preserve">Titel + Einstiegsfrage</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wer wir sind</t>
   </si>
   <si>
@@ -125,28 +128,28 @@
     <t xml:space="preserve">Produziert, angeboten, verkauft</t>
   </si>
   <si>
-    <t xml:space="preserve">Warum wir so entschieden haben</t>
+    <t xml:space="preserve">Drei Entscheidungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zwei Kennzahlen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wirtschaftlichkeit &amp; Schlussbestand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkaufswert</t>
   </si>
   <si>
     <t xml:space="preserve">Wirtschaftsdienst</t>
   </si>
   <si>
-    <t xml:space="preserve">Unsere Kennzahlen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wirtschaftlichkeit &amp; Schlussbestand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkaufswert</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reflexion</t>
   </si>
   <si>
     <t xml:space="preserve">Bezug zur Gründung</t>
   </si>
   <si>
-    <t xml:space="preserve">Vielen Dank</t>
+    <t xml:space="preserve">Schluss + Danke</t>
   </si>
   <si>
     <t xml:space="preserve">Zeit pro Person</t>
@@ -961,11 +964,11 @@
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="12" t="n">
-        <v>0.000231481481481482</v>
+        <v>0.000405092592592593</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -973,7 +976,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="12" t="n">
@@ -985,11 +988,11 @@
         <v>3</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="12" t="n">
-        <v>0.000520833333333333</v>
+        <v>0.000462962962962963</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -997,7 +1000,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="12" t="n">
@@ -1009,11 +1012,11 @@
         <v>5</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="12" t="n">
-        <v>0.000752314814814815</v>
+        <v>0.000810185185185185</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1021,11 +1024,11 @@
         <v>6</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="12" t="n">
-        <v>0.000578703703703704</v>
+        <v>0.000694444444444445</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1033,11 +1036,11 @@
         <v>7</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="12" t="n">
-        <v>0.000694444444444445</v>
+        <v>0.000578703703703704</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1045,11 +1048,11 @@
         <v>8</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="12" t="n">
-        <v>0.000636574074074074</v>
+        <v>0.000578703703703704</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1057,7 +1060,7 @@
         <v>9</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="12" t="n">
@@ -1069,11 +1072,11 @@
         <v>10</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="12" t="n">
-        <v>0.000925925925925926</v>
+        <v>0.000810185185185185</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1081,11 +1084,11 @@
         <v>11</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="12" t="n">
-        <v>0.000810185185185185</v>
+        <v>0.000752314814814815</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1093,16 +1096,16 @@
         <v>12</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="12" t="n">
-        <v>0.000115740740740741</v>
+        <v>0.000347222222222222</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,16 +1146,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D23" s="16" t="n">
         <f aca="false">SUM(E5:E16)</f>
-        <v>0.00706018518518519</v>
+        <v>0.0072337962962963</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C24" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D24" s="18" t="str">
         <f aca="false">COUNTBLANK(D5:D16)&amp;" Folien"</f>

</xml_diff>